<commit_message>
Edited Mapping for Atherosklerotisches Erstereignis
</commit_message>
<xml_diff>
--- a/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_alpha3.xlsx
+++ b/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_alpha3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tmfev.sharepoint.com/sites/tmf/mi-i/Taskforce Kerndatensatz/04_Erweiterungsmodule/Modul_Kardiologie/03 Datensatz/Acribis-FHIR_Mapping-Hilfe/Überarbeitung zu Alpha3-Release_Juni26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M3nthos\Desktop\git-projects\kerndatensatz-kardiologie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="14_{D828A212-3488-4D58-A0EA-B96B24CFDD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D67128D-51C9-475F-83F6-EE1D21491CD6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB0027C-68F3-4087-914D-ECA0D381F7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="30" windowWidth="38370" windowHeight="20850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Legende" sheetId="9" r:id="rId1"/>
@@ -11370,20 +11370,6 @@
     </r>
   </si>
   <si>
-    <t>Aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-vs-kardio-atherosklerotisches-ereignis-snomedct
-53741008 "Coronary arteriosclerosis (disorder)"
-399957001 "Peripheral arterial occlusive disease (disorder)"
-233985008 "Abdominal aortic aneurysm (disorder)"	
-232035005 "Retinal artery occlusion (disorder)" = dt. Zentralarterienverschluss
-422504002 "Ischemic stroke (disorder)"
-88032003 "Amaurosis fugax (disorder)"
-266257000 "Transient ischemic attack (disorder)"
-1287902001 "Operation on carotid artery (procedure)"
-Falls nicht genauer bekannt: 
-ae &lt;=&gt; "Atherosklerotisches Ereignis"
-aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-cs-kardio-atherosklerotisches-ereignis</t>
-  </si>
-  <si>
     <t>keine, siehe Modul Studie IG oder Modul Consent IG</t>
   </si>
   <si>
@@ -12179,6 +12165,20 @@
 Unknown if ever smoked = LA18980-5
 Falls die Rauchmenge dokumentiert wurde, kann bei &gt;20 Zigaretten pro Tag auf einen starken Raucher geschlossen werden.
 Heavy tobacco smoker = LA18981-3</t>
+  </si>
+  <si>
+    <t>Aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-vs-kardio-atherosklerotisches-ereignis-snomedct
+53741008 "Coronary arteriosclerosis (disorder)"
+399957001 "Peripheral arterial occlusive disease (disorder)"
+233985008 "Abdominal aortic aneurysm (disorder)"	
+232035005 "Retinal artery occlusion (disorder)" = dt. Zentralarterienverschluss
+422504002 "Ischemic stroke (disorder)"
+88032003 "Amaurosis fugax (disorder)"
+266257000 "Transient ischemic attack (disorder)"
+1287902001 "Operation on carotid artery (procedure)"
+Falls nicht genauer bekannt: 
+ae &lt;=&gt; "Atherosklerotisches Ereignis" oder falls aus Item 67 bekannt, dann "eg-cv"
+aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-cs-kardio-atherosklerotisches-ereignis</t>
   </si>
 </sst>
 </file>
@@ -13044,19 +13044,19 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -15211,7 +15211,7 @@
         <v>2426</v>
       </c>
       <c r="P2" s="56" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="Q2" s="89" t="s">
         <v>2548</v>
@@ -15239,7 +15239,7 @@
       </c>
       <c r="J3" s="56"/>
       <c r="K3" s="96" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="L3" s="97" t="s">
         <v>2513</v>
@@ -15785,7 +15785,7 @@
         <v>2465</v>
       </c>
       <c r="P14" s="55" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="Q14" s="68"/>
     </row>
@@ -15924,7 +15924,7 @@
       </c>
       <c r="O17" s="58"/>
       <c r="P17" s="56" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="Q17" s="2"/>
     </row>
@@ -16345,7 +16345,7 @@
       <c r="P26" s="58"/>
       <c r="Q26" s="2"/>
     </row>
-    <row r="27" spans="1:17" ht="375">
+    <row r="27" spans="1:17" ht="390">
       <c r="A27" s="95" t="s">
         <v>205</v>
       </c>
@@ -16386,7 +16386,7 @@
         <v>212</v>
       </c>
       <c r="N27" s="96" t="s">
-        <v>2681</v>
+        <v>2696</v>
       </c>
       <c r="O27" s="96" t="s">
         <v>213</v>
@@ -16690,19 +16690,19 @@
         <v>257</v>
       </c>
       <c r="K34" s="104" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="L34" s="101" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="M34" s="55" t="s">
         <v>212</v>
       </c>
       <c r="N34" s="55" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="O34" s="56" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
       <c r="P34" s="58"/>
       <c r="Q34" s="2"/>
@@ -16739,7 +16739,7 @@
         <v>263</v>
       </c>
       <c r="K35" s="56" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="L35" s="101" t="s">
         <v>2506</v>
@@ -16786,7 +16786,7 @@
         <v>2424</v>
       </c>
       <c r="K36" s="56" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="L36" s="101" t="s">
         <v>2506</v>
@@ -16835,7 +16835,7 @@
         <v>271</v>
       </c>
       <c r="K37" s="56" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="L37" s="101" t="s">
         <v>2506</v>
@@ -16884,7 +16884,7 @@
         <v>283</v>
       </c>
       <c r="K38" s="56" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="L38" s="101" t="s">
         <v>284</v>
@@ -16933,7 +16933,7 @@
         <v>2425</v>
       </c>
       <c r="K39" s="56" t="s">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="L39" s="101" t="s">
         <v>2515</v>
@@ -16945,10 +16945,10 @@
         <v>293</v>
       </c>
       <c r="O39" s="114" t="s">
+        <v>2687</v>
+      </c>
+      <c r="P39" s="56" t="s">
         <v>2688</v>
-      </c>
-      <c r="P39" s="56" t="s">
-        <v>2689</v>
       </c>
       <c r="Q39" s="2"/>
     </row>
@@ -25317,10 +25317,10 @@
       <c r="E2" s="43" t="s">
         <v>1194</v>
       </c>
-      <c r="F2" s="120" t="s">
+      <c r="F2" s="119" t="s">
         <v>1195</v>
       </c>
-      <c r="G2" s="120"/>
+      <c r="G2" s="119"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="43"/>
@@ -25394,10 +25394,10 @@
       <c r="E7" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F7" s="121" t="s">
+      <c r="F7" s="120" t="s">
         <v>1205</v>
       </c>
-      <c r="G7" s="117"/>
+      <c r="G7" s="116"/>
     </row>
     <row r="8" spans="1:7" s="44" customFormat="1">
       <c r="D8" s="44" t="s">
@@ -25406,8 +25406,8 @@
       <c r="E8" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F8" s="121"/>
-      <c r="G8" s="117"/>
+      <c r="F8" s="120"/>
+      <c r="G8" s="116"/>
     </row>
     <row r="9" spans="1:7" s="44" customFormat="1">
       <c r="D9" s="44" t="s">
@@ -25416,8 +25416,8 @@
       <c r="E9" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F9" s="121"/>
-      <c r="G9" s="117"/>
+      <c r="F9" s="120"/>
+      <c r="G9" s="116"/>
     </row>
     <row r="10" spans="1:7" s="44" customFormat="1">
       <c r="D10" s="44" t="s">
@@ -25426,8 +25426,8 @@
       <c r="E10" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F10" s="121"/>
-      <c r="G10" s="117"/>
+      <c r="F10" s="120"/>
+      <c r="G10" s="116"/>
     </row>
     <row r="11" spans="1:7" s="44" customFormat="1">
       <c r="B11" s="44" t="s">
@@ -25442,8 +25442,8 @@
       <c r="E11" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F11" s="121"/>
-      <c r="G11" s="117"/>
+      <c r="F11" s="120"/>
+      <c r="G11" s="116"/>
     </row>
     <row r="12" spans="1:7" s="44" customFormat="1">
       <c r="B12" s="44" t="s">
@@ -25452,8 +25452,8 @@
       <c r="C12" s="44" t="s">
         <v>1207</v>
       </c>
-      <c r="F12" s="121"/>
-      <c r="G12" s="117"/>
+      <c r="F12" s="120"/>
+      <c r="G12" s="116"/>
     </row>
     <row r="13" spans="1:7" s="44" customFormat="1">
       <c r="B13" s="44" t="s">
@@ -25462,8 +25462,8 @@
       <c r="C13" s="44" t="s">
         <v>1209</v>
       </c>
-      <c r="F13" s="121"/>
-      <c r="G13" s="117"/>
+      <c r="F13" s="120"/>
+      <c r="G13" s="116"/>
     </row>
     <row r="14" spans="1:7" s="43" customFormat="1">
       <c r="A14" s="43" t="s">
@@ -25475,7 +25475,7 @@
       <c r="C14" s="43" t="s">
         <v>1197</v>
       </c>
-      <c r="F14" s="122" t="s">
+      <c r="F14" s="121" t="s">
         <v>1211</v>
       </c>
       <c r="G14" s="118" t="s">
@@ -25534,10 +25534,10 @@
       </c>
       <c r="D19" s="44"/>
       <c r="E19" s="44"/>
-      <c r="F19" s="116" t="s">
+      <c r="F19" s="122" t="s">
         <v>1195</v>
       </c>
-      <c r="G19" s="117"/>
+      <c r="G19" s="116"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="44"/>
@@ -25549,8 +25549,8 @@
       </c>
       <c r="D20" s="44"/>
       <c r="E20" s="44"/>
-      <c r="F20" s="117"/>
-      <c r="G20" s="117"/>
+      <c r="F20" s="116"/>
+      <c r="G20" s="116"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="44"/>
@@ -25562,8 +25562,8 @@
       </c>
       <c r="D21" s="44"/>
       <c r="E21" s="44"/>
-      <c r="F21" s="117"/>
-      <c r="G21" s="117"/>
+      <c r="F21" s="116"/>
+      <c r="G21" s="116"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="44"/>
@@ -25575,8 +25575,8 @@
       </c>
       <c r="D22" s="44"/>
       <c r="E22" s="44"/>
-      <c r="F22" s="117"/>
-      <c r="G22" s="117"/>
+      <c r="F22" s="116"/>
+      <c r="G22" s="116"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="44"/>
@@ -25588,8 +25588,8 @@
       </c>
       <c r="D23" s="44"/>
       <c r="E23" s="44"/>
-      <c r="F23" s="117"/>
-      <c r="G23" s="117"/>
+      <c r="F23" s="116"/>
+      <c r="G23" s="116"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="43" t="s">
@@ -25622,10 +25622,10 @@
       </c>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
-      <c r="F25" s="117" t="s">
+      <c r="F25" s="116" t="s">
         <v>1195</v>
       </c>
-      <c r="G25" s="119"/>
+      <c r="G25" s="123"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="44"/>
@@ -25637,8 +25637,8 @@
       </c>
       <c r="D26" s="44"/>
       <c r="E26" s="44"/>
-      <c r="F26" s="117"/>
-      <c r="G26" s="119"/>
+      <c r="F26" s="116"/>
+      <c r="G26" s="123"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="44"/>
@@ -25650,8 +25650,8 @@
       </c>
       <c r="D27" s="44"/>
       <c r="E27" s="44"/>
-      <c r="F27" s="117"/>
-      <c r="G27" s="119"/>
+      <c r="F27" s="116"/>
+      <c r="G27" s="123"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="44"/>
@@ -25663,8 +25663,8 @@
       </c>
       <c r="D28" s="44"/>
       <c r="E28" s="44"/>
-      <c r="F28" s="117"/>
-      <c r="G28" s="119"/>
+      <c r="F28" s="116"/>
+      <c r="G28" s="123"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="44"/>
@@ -25676,8 +25676,8 @@
       </c>
       <c r="D29" s="44"/>
       <c r="E29" s="44"/>
-      <c r="F29" s="117"/>
-      <c r="G29" s="119"/>
+      <c r="F29" s="116"/>
+      <c r="G29" s="123"/>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="44"/>
@@ -25689,8 +25689,8 @@
       </c>
       <c r="D30" s="44"/>
       <c r="E30" s="44"/>
-      <c r="F30" s="117"/>
-      <c r="G30" s="119"/>
+      <c r="F30" s="116"/>
+      <c r="G30" s="123"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="44"/>
@@ -25702,8 +25702,8 @@
       </c>
       <c r="D31" s="44"/>
       <c r="E31" s="44"/>
-      <c r="F31" s="117"/>
-      <c r="G31" s="119"/>
+      <c r="F31" s="116"/>
+      <c r="G31" s="123"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="43" t="s">
@@ -26141,10 +26141,10 @@
       </c>
       <c r="D64" s="44"/>
       <c r="E64" s="44"/>
-      <c r="F64" s="117" t="s">
+      <c r="F64" s="116" t="s">
         <v>1306</v>
       </c>
-      <c r="G64" s="117"/>
+      <c r="G64" s="116"/>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="44"/>
@@ -26156,8 +26156,8 @@
       <c r="E65" s="44" t="s">
         <v>1308</v>
       </c>
-      <c r="F65" s="117"/>
-      <c r="G65" s="117"/>
+      <c r="F65" s="116"/>
+      <c r="G65" s="116"/>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" s="44"/>
@@ -26169,8 +26169,8 @@
       <c r="E66" s="44" t="s">
         <v>1310</v>
       </c>
-      <c r="F66" s="117"/>
-      <c r="G66" s="117"/>
+      <c r="F66" s="116"/>
+      <c r="G66" s="116"/>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="44"/>
@@ -26182,8 +26182,8 @@
       </c>
       <c r="D67" s="44"/>
       <c r="E67" s="44"/>
-      <c r="F67" s="117"/>
-      <c r="G67" s="117"/>
+      <c r="F67" s="116"/>
+      <c r="G67" s="116"/>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" s="44"/>
@@ -26195,8 +26195,8 @@
       <c r="E68" s="44" t="s">
         <v>1314</v>
       </c>
-      <c r="F68" s="117"/>
-      <c r="G68" s="117"/>
+      <c r="F68" s="116"/>
+      <c r="G68" s="116"/>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="44"/>
@@ -26212,8 +26212,8 @@
       <c r="E69" s="44" t="s">
         <v>1318</v>
       </c>
-      <c r="F69" s="117"/>
-      <c r="G69" s="117"/>
+      <c r="F69" s="116"/>
+      <c r="G69" s="116"/>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="44"/>
@@ -26225,8 +26225,8 @@
       <c r="E70" s="44" t="s">
         <v>1320</v>
       </c>
-      <c r="F70" s="117"/>
-      <c r="G70" s="117"/>
+      <c r="F70" s="116"/>
+      <c r="G70" s="116"/>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="44"/>
@@ -26238,8 +26238,8 @@
       <c r="E71" s="44" t="s">
         <v>1322</v>
       </c>
-      <c r="F71" s="117"/>
-      <c r="G71" s="117"/>
+      <c r="F71" s="116"/>
+      <c r="G71" s="116"/>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="44"/>
@@ -26251,8 +26251,8 @@
       <c r="E72" s="44" t="s">
         <v>1324</v>
       </c>
-      <c r="F72" s="117"/>
-      <c r="G72" s="117"/>
+      <c r="F72" s="116"/>
+      <c r="G72" s="116"/>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="44"/>
@@ -26264,8 +26264,8 @@
       <c r="E73" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F73" s="117"/>
-      <c r="G73" s="117"/>
+      <c r="F73" s="116"/>
+      <c r="G73" s="116"/>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" s="44"/>
@@ -26277,8 +26277,8 @@
       </c>
       <c r="D74" s="44"/>
       <c r="E74" s="44"/>
-      <c r="F74" s="117"/>
-      <c r="G74" s="117"/>
+      <c r="F74" s="116"/>
+      <c r="G74" s="116"/>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="44"/>
@@ -26290,8 +26290,8 @@
       <c r="E75" s="44" t="s">
         <v>1330</v>
       </c>
-      <c r="F75" s="117"/>
-      <c r="G75" s="117"/>
+      <c r="F75" s="116"/>
+      <c r="G75" s="116"/>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" s="44"/>
@@ -26307,8 +26307,8 @@
       <c r="E76" s="44" t="s">
         <v>1334</v>
       </c>
-      <c r="F76" s="117"/>
-      <c r="G76" s="117"/>
+      <c r="F76" s="116"/>
+      <c r="G76" s="116"/>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="44"/>
@@ -26320,8 +26320,8 @@
       <c r="E77" s="44" t="s">
         <v>1336</v>
       </c>
-      <c r="F77" s="117"/>
-      <c r="G77" s="117"/>
+      <c r="F77" s="116"/>
+      <c r="G77" s="116"/>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" s="44"/>
@@ -26333,8 +26333,8 @@
       <c r="E78" s="44" t="s">
         <v>1338</v>
       </c>
-      <c r="F78" s="117"/>
-      <c r="G78" s="117"/>
+      <c r="F78" s="116"/>
+      <c r="G78" s="116"/>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="44"/>
@@ -26346,8 +26346,8 @@
       <c r="E79" s="44" t="s">
         <v>1340</v>
       </c>
-      <c r="F79" s="117"/>
-      <c r="G79" s="117"/>
+      <c r="F79" s="116"/>
+      <c r="G79" s="116"/>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" s="44"/>
@@ -26359,8 +26359,8 @@
       <c r="E80" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F80" s="117"/>
-      <c r="G80" s="117"/>
+      <c r="F80" s="116"/>
+      <c r="G80" s="116"/>
     </row>
     <row r="81" spans="1:7">
       <c r="A81" s="44"/>
@@ -26376,8 +26376,8 @@
       <c r="E81" s="44" t="s">
         <v>1346</v>
       </c>
-      <c r="F81" s="117"/>
-      <c r="G81" s="117"/>
+      <c r="F81" s="116"/>
+      <c r="G81" s="116"/>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" s="44"/>
@@ -26389,8 +26389,8 @@
       <c r="E82" s="44" t="s">
         <v>1348</v>
       </c>
-      <c r="F82" s="117"/>
-      <c r="G82" s="117"/>
+      <c r="F82" s="116"/>
+      <c r="G82" s="116"/>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="44"/>
@@ -26402,8 +26402,8 @@
       <c r="E83" s="44" t="s">
         <v>1350</v>
       </c>
-      <c r="F83" s="117"/>
-      <c r="G83" s="117"/>
+      <c r="F83" s="116"/>
+      <c r="G83" s="116"/>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" s="44"/>
@@ -26415,8 +26415,8 @@
       </c>
       <c r="D84" s="44"/>
       <c r="E84" s="44"/>
-      <c r="F84" s="117"/>
-      <c r="G84" s="117"/>
+      <c r="F84" s="116"/>
+      <c r="G84" s="116"/>
     </row>
     <row r="85" spans="1:7">
       <c r="A85" s="44"/>
@@ -26428,8 +26428,8 @@
       <c r="E85" s="44" t="s">
         <v>1354</v>
       </c>
-      <c r="F85" s="117"/>
-      <c r="G85" s="117"/>
+      <c r="F85" s="116"/>
+      <c r="G85" s="116"/>
     </row>
     <row r="86" spans="1:7">
       <c r="A86" s="44"/>
@@ -26441,8 +26441,8 @@
       <c r="E86" s="44" t="s">
         <v>1356</v>
       </c>
-      <c r="F86" s="117"/>
-      <c r="G86" s="117"/>
+      <c r="F86" s="116"/>
+      <c r="G86" s="116"/>
     </row>
     <row r="87" spans="1:7">
       <c r="A87" s="44"/>
@@ -26454,8 +26454,8 @@
       <c r="E87" s="44" t="s">
         <v>1358</v>
       </c>
-      <c r="F87" s="117"/>
-      <c r="G87" s="117"/>
+      <c r="F87" s="116"/>
+      <c r="G87" s="116"/>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="44"/>
@@ -26467,8 +26467,8 @@
       </c>
       <c r="D88" s="44"/>
       <c r="E88" s="44"/>
-      <c r="F88" s="117"/>
-      <c r="G88" s="117"/>
+      <c r="F88" s="116"/>
+      <c r="G88" s="116"/>
     </row>
     <row r="89" spans="1:7">
       <c r="A89" s="43" t="s">
@@ -26499,10 +26499,10 @@
       </c>
       <c r="D90" s="44"/>
       <c r="E90" s="44"/>
-      <c r="F90" s="117" t="s">
+      <c r="F90" s="116" t="s">
         <v>1364</v>
       </c>
-      <c r="G90" s="117"/>
+      <c r="G90" s="116"/>
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="44"/>
@@ -26514,8 +26514,8 @@
       </c>
       <c r="D91" s="44"/>
       <c r="E91" s="44"/>
-      <c r="F91" s="117"/>
-      <c r="G91" s="117"/>
+      <c r="F91" s="116"/>
+      <c r="G91" s="116"/>
     </row>
     <row r="92" spans="1:7">
       <c r="A92" s="44"/>
@@ -26527,8 +26527,8 @@
       <c r="E92" s="44" t="s">
         <v>1368</v>
       </c>
-      <c r="F92" s="117"/>
-      <c r="G92" s="117"/>
+      <c r="F92" s="116"/>
+      <c r="G92" s="116"/>
     </row>
     <row r="93" spans="1:7">
       <c r="A93" s="44"/>
@@ -26540,8 +26540,8 @@
       </c>
       <c r="D93" s="44"/>
       <c r="E93" s="44"/>
-      <c r="F93" s="117"/>
-      <c r="G93" s="117"/>
+      <c r="F93" s="116"/>
+      <c r="G93" s="116"/>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="44"/>
@@ -26553,8 +26553,8 @@
       </c>
       <c r="D94" s="44"/>
       <c r="E94" s="44"/>
-      <c r="F94" s="117"/>
-      <c r="G94" s="117"/>
+      <c r="F94" s="116"/>
+      <c r="G94" s="116"/>
     </row>
     <row r="95" spans="1:7">
       <c r="A95" s="44"/>
@@ -26566,8 +26566,8 @@
       <c r="E95" s="44" t="s">
         <v>1374</v>
       </c>
-      <c r="F95" s="117"/>
-      <c r="G95" s="117"/>
+      <c r="F95" s="116"/>
+      <c r="G95" s="116"/>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" s="44"/>
@@ -26579,8 +26579,8 @@
       <c r="E96" s="44" t="s">
         <v>1376</v>
       </c>
-      <c r="F96" s="117"/>
-      <c r="G96" s="117"/>
+      <c r="F96" s="116"/>
+      <c r="G96" s="116"/>
     </row>
     <row r="97" spans="1:7">
       <c r="A97" s="44"/>
@@ -26592,8 +26592,8 @@
       <c r="E97" s="44" t="s">
         <v>1378</v>
       </c>
-      <c r="F97" s="117"/>
-      <c r="G97" s="117"/>
+      <c r="F97" s="116"/>
+      <c r="G97" s="116"/>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="44"/>
@@ -26605,8 +26605,8 @@
       <c r="E98" s="44" t="s">
         <v>1380</v>
       </c>
-      <c r="F98" s="117"/>
-      <c r="G98" s="117"/>
+      <c r="F98" s="116"/>
+      <c r="G98" s="116"/>
     </row>
     <row r="99" spans="1:7">
       <c r="A99" s="44"/>
@@ -26618,8 +26618,8 @@
       </c>
       <c r="D99" s="44"/>
       <c r="E99" s="44"/>
-      <c r="F99" s="117"/>
-      <c r="G99" s="117"/>
+      <c r="F99" s="116"/>
+      <c r="G99" s="116"/>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="44"/>
@@ -26631,8 +26631,8 @@
       <c r="E100" s="44" t="s">
         <v>1384</v>
       </c>
-      <c r="F100" s="117"/>
-      <c r="G100" s="117"/>
+      <c r="F100" s="116"/>
+      <c r="G100" s="116"/>
     </row>
     <row r="101" spans="1:7">
       <c r="A101" s="44"/>
@@ -26644,8 +26644,8 @@
       <c r="E101" s="44" t="s">
         <v>1386</v>
       </c>
-      <c r="F101" s="117"/>
-      <c r="G101" s="117"/>
+      <c r="F101" s="116"/>
+      <c r="G101" s="116"/>
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="44"/>
@@ -26657,8 +26657,8 @@
       </c>
       <c r="D102" s="44"/>
       <c r="E102" s="44"/>
-      <c r="F102" s="117"/>
-      <c r="G102" s="117"/>
+      <c r="F102" s="116"/>
+      <c r="G102" s="116"/>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="44"/>
@@ -26670,8 +26670,8 @@
       </c>
       <c r="D103" s="44"/>
       <c r="E103" s="44"/>
-      <c r="F103" s="117"/>
-      <c r="G103" s="117"/>
+      <c r="F103" s="116"/>
+      <c r="G103" s="116"/>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="44"/>
@@ -26683,8 +26683,8 @@
       <c r="E104" s="44" t="s">
         <v>1392</v>
       </c>
-      <c r="F104" s="117"/>
-      <c r="G104" s="117"/>
+      <c r="F104" s="116"/>
+      <c r="G104" s="116"/>
     </row>
     <row r="105" spans="1:7">
       <c r="A105" s="44"/>
@@ -26696,8 +26696,8 @@
       <c r="E105" s="44" t="s">
         <v>1394</v>
       </c>
-      <c r="F105" s="117"/>
-      <c r="G105" s="117"/>
+      <c r="F105" s="116"/>
+      <c r="G105" s="116"/>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" s="44"/>
@@ -26709,8 +26709,8 @@
       <c r="E106" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F106" s="117"/>
-      <c r="G106" s="117"/>
+      <c r="F106" s="116"/>
+      <c r="G106" s="116"/>
     </row>
     <row r="107" spans="1:7">
       <c r="A107" s="44"/>
@@ -26722,8 +26722,8 @@
       <c r="E107" s="44" t="s">
         <v>1279</v>
       </c>
-      <c r="F107" s="117"/>
-      <c r="G107" s="117"/>
+      <c r="F107" s="116"/>
+      <c r="G107" s="116"/>
     </row>
     <row r="108" spans="1:7">
       <c r="A108" s="44"/>
@@ -26735,8 +26735,8 @@
       </c>
       <c r="D108" s="44"/>
       <c r="E108" s="44"/>
-      <c r="F108" s="117"/>
-      <c r="G108" s="117"/>
+      <c r="F108" s="116"/>
+      <c r="G108" s="116"/>
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="44"/>
@@ -26748,8 +26748,8 @@
       </c>
       <c r="D109" s="44"/>
       <c r="E109" s="44"/>
-      <c r="F109" s="117"/>
-      <c r="G109" s="117"/>
+      <c r="F109" s="116"/>
+      <c r="G109" s="116"/>
     </row>
     <row r="110" spans="1:7">
       <c r="A110" s="44"/>
@@ -26761,8 +26761,8 @@
       </c>
       <c r="D110" s="44"/>
       <c r="E110" s="44"/>
-      <c r="F110" s="117"/>
-      <c r="G110" s="117"/>
+      <c r="F110" s="116"/>
+      <c r="G110" s="116"/>
     </row>
     <row r="111" spans="1:7">
       <c r="A111" s="44"/>
@@ -26774,8 +26774,8 @@
       </c>
       <c r="D111" s="44"/>
       <c r="E111" s="44"/>
-      <c r="F111" s="117"/>
-      <c r="G111" s="117"/>
+      <c r="F111" s="116"/>
+      <c r="G111" s="116"/>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="44"/>
@@ -26787,8 +26787,8 @@
       </c>
       <c r="D112" s="44"/>
       <c r="E112" s="44"/>
-      <c r="F112" s="117"/>
-      <c r="G112" s="117"/>
+      <c r="F112" s="116"/>
+      <c r="G112" s="116"/>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="43" t="s">
@@ -26875,10 +26875,10 @@
       <c r="E118" s="44" t="s">
         <v>1419</v>
       </c>
-      <c r="F118" s="117" t="s">
+      <c r="F118" s="116" t="s">
         <v>1420</v>
       </c>
-      <c r="G118" s="117"/>
+      <c r="G118" s="116"/>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="44"/>
@@ -26894,8 +26894,8 @@
       <c r="E119" s="44" t="s">
         <v>1424</v>
       </c>
-      <c r="F119" s="117"/>
-      <c r="G119" s="117"/>
+      <c r="F119" s="116"/>
+      <c r="G119" s="116"/>
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
@@ -28380,10 +28380,10 @@
       </c>
       <c r="D279" s="44"/>
       <c r="E279" s="44"/>
-      <c r="F279" s="117" t="s">
+      <c r="F279" s="116" t="s">
         <v>1687</v>
       </c>
-      <c r="G279" s="117"/>
+      <c r="G279" s="116"/>
     </row>
     <row r="280" spans="1:7">
       <c r="A280" s="44"/>
@@ -28395,8 +28395,8 @@
       <c r="E280" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F280" s="117"/>
-      <c r="G280" s="117"/>
+      <c r="F280" s="116"/>
+      <c r="G280" s="116"/>
     </row>
     <row r="281" spans="1:7">
       <c r="A281" s="44"/>
@@ -28408,8 +28408,8 @@
       </c>
       <c r="D281" s="44"/>
       <c r="E281" s="44"/>
-      <c r="F281" s="117"/>
-      <c r="G281" s="117"/>
+      <c r="F281" s="116"/>
+      <c r="G281" s="116"/>
     </row>
     <row r="282" spans="1:7">
       <c r="A282" s="44"/>
@@ -28425,8 +28425,8 @@
       <c r="E282" s="44" t="s">
         <v>1695</v>
       </c>
-      <c r="F282" s="117"/>
-      <c r="G282" s="117"/>
+      <c r="F282" s="116"/>
+      <c r="G282" s="116"/>
     </row>
     <row r="283" spans="1:7">
       <c r="A283" s="44"/>
@@ -28438,8 +28438,8 @@
       </c>
       <c r="D283" s="44"/>
       <c r="E283" s="44"/>
-      <c r="F283" s="117"/>
-      <c r="G283" s="117"/>
+      <c r="F283" s="116"/>
+      <c r="G283" s="116"/>
     </row>
     <row r="284" spans="1:7">
       <c r="A284" s="44"/>
@@ -28455,8 +28455,8 @@
       <c r="E284" s="44" t="s">
         <v>1701</v>
       </c>
-      <c r="F284" s="117"/>
-      <c r="G284" s="117"/>
+      <c r="F284" s="116"/>
+      <c r="G284" s="116"/>
     </row>
     <row r="285" spans="1:7">
       <c r="A285" s="44"/>
@@ -28468,8 +28468,8 @@
       <c r="E285" s="44" t="s">
         <v>1567</v>
       </c>
-      <c r="F285" s="117"/>
-      <c r="G285" s="117"/>
+      <c r="F285" s="116"/>
+      <c r="G285" s="116"/>
     </row>
     <row r="286" spans="1:7">
       <c r="A286" s="44"/>
@@ -28481,8 +28481,8 @@
       <c r="E286" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F286" s="117"/>
-      <c r="G286" s="117"/>
+      <c r="F286" s="116"/>
+      <c r="G286" s="116"/>
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="44"/>
@@ -28494,8 +28494,8 @@
       <c r="E287" s="44" t="s">
         <v>1265</v>
       </c>
-      <c r="F287" s="117"/>
-      <c r="G287" s="117"/>
+      <c r="F287" s="116"/>
+      <c r="G287" s="116"/>
     </row>
     <row r="288" spans="1:7">
       <c r="A288" s="44"/>
@@ -28507,8 +28507,8 @@
       <c r="E288" s="44" t="s">
         <v>1281</v>
       </c>
-      <c r="F288" s="117"/>
-      <c r="G288" s="117"/>
+      <c r="F288" s="116"/>
+      <c r="G288" s="116"/>
     </row>
     <row r="289" spans="1:7">
       <c r="A289" s="44"/>
@@ -28520,8 +28520,8 @@
       <c r="E289" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F289" s="117"/>
-      <c r="G289" s="117"/>
+      <c r="F289" s="116"/>
+      <c r="G289" s="116"/>
     </row>
     <row r="290" spans="1:7">
       <c r="A290" s="44"/>
@@ -28533,8 +28533,8 @@
       </c>
       <c r="D290" s="44"/>
       <c r="E290" s="44"/>
-      <c r="F290" s="117"/>
-      <c r="G290" s="117"/>
+      <c r="F290" s="116"/>
+      <c r="G290" s="116"/>
     </row>
     <row r="291" spans="1:7">
       <c r="A291" s="44"/>
@@ -28546,8 +28546,8 @@
       <c r="E291" s="44" t="s">
         <v>1705</v>
       </c>
-      <c r="F291" s="117"/>
-      <c r="G291" s="117"/>
+      <c r="F291" s="116"/>
+      <c r="G291" s="116"/>
     </row>
     <row r="292" spans="1:7">
       <c r="A292" s="44"/>
@@ -28559,8 +28559,8 @@
       <c r="E292" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F292" s="117"/>
-      <c r="G292" s="117"/>
+      <c r="F292" s="116"/>
+      <c r="G292" s="116"/>
     </row>
     <row r="293" spans="1:7">
       <c r="A293" s="44"/>
@@ -28572,8 +28572,8 @@
       <c r="E293" s="44" t="s">
         <v>1571</v>
       </c>
-      <c r="F293" s="117"/>
-      <c r="G293" s="117"/>
+      <c r="F293" s="116"/>
+      <c r="G293" s="116"/>
     </row>
     <row r="294" spans="1:7">
       <c r="A294" s="44"/>
@@ -28585,8 +28585,8 @@
       <c r="E294" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F294" s="117"/>
-      <c r="G294" s="117"/>
+      <c r="F294" s="116"/>
+      <c r="G294" s="116"/>
     </row>
     <row r="295" spans="1:7">
       <c r="A295" s="44"/>
@@ -28598,8 +28598,8 @@
       </c>
       <c r="D295" s="44"/>
       <c r="E295" s="44"/>
-      <c r="F295" s="117"/>
-      <c r="G295" s="117"/>
+      <c r="F295" s="116"/>
+      <c r="G295" s="116"/>
     </row>
     <row r="296" spans="1:7">
       <c r="A296" s="43" t="s">
@@ -28701,10 +28701,10 @@
       </c>
       <c r="D302" s="44"/>
       <c r="E302" s="44"/>
-      <c r="F302" s="117" t="s">
+      <c r="F302" s="116" t="s">
         <v>1711</v>
       </c>
-      <c r="G302" s="117" t="s">
+      <c r="G302" s="116" t="s">
         <v>1712</v>
       </c>
     </row>
@@ -28718,8 +28718,8 @@
       <c r="E303" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F303" s="117"/>
-      <c r="G303" s="117"/>
+      <c r="F303" s="116"/>
+      <c r="G303" s="116"/>
     </row>
     <row r="304" spans="1:7">
       <c r="A304" s="43" t="s">
@@ -28925,10 +28925,10 @@
       </c>
       <c r="D316" s="44"/>
       <c r="E316" s="44"/>
-      <c r="F316" s="117" t="s">
+      <c r="F316" s="116" t="s">
         <v>1729</v>
       </c>
-      <c r="G316" s="117"/>
+      <c r="G316" s="116"/>
     </row>
     <row r="317" spans="1:7">
       <c r="A317" s="44"/>
@@ -28940,8 +28940,8 @@
       </c>
       <c r="D317" s="44"/>
       <c r="E317" s="44"/>
-      <c r="F317" s="117"/>
-      <c r="G317" s="117"/>
+      <c r="F317" s="116"/>
+      <c r="G317" s="116"/>
     </row>
     <row r="318" spans="1:7">
       <c r="A318" s="44"/>
@@ -28953,8 +28953,8 @@
       </c>
       <c r="D318" s="44"/>
       <c r="E318" s="44"/>
-      <c r="F318" s="117"/>
-      <c r="G318" s="117"/>
+      <c r="F318" s="116"/>
+      <c r="G318" s="116"/>
     </row>
     <row r="319" spans="1:7">
       <c r="A319" t="s">
@@ -30175,10 +30175,10 @@
       <c r="E450" s="44" t="s">
         <v>1981</v>
       </c>
-      <c r="F450" s="123" t="s">
+      <c r="F450" s="117" t="s">
         <v>1982</v>
       </c>
-      <c r="G450" s="117"/>
+      <c r="G450" s="116"/>
     </row>
     <row r="451" spans="1:7">
       <c r="A451" s="44"/>
@@ -30190,8 +30190,8 @@
       </c>
       <c r="D451" s="44"/>
       <c r="E451" s="44"/>
-      <c r="F451" s="123"/>
-      <c r="G451" s="117"/>
+      <c r="F451" s="117"/>
+      <c r="G451" s="116"/>
     </row>
     <row r="452" spans="1:7">
       <c r="A452" s="44"/>
@@ -30207,8 +30207,8 @@
       <c r="E452" s="44" t="s">
         <v>1988</v>
       </c>
-      <c r="F452" s="123"/>
-      <c r="G452" s="117"/>
+      <c r="F452" s="117"/>
+      <c r="G452" s="116"/>
     </row>
     <row r="453" spans="1:7">
       <c r="A453" s="44"/>
@@ -30220,8 +30220,8 @@
       <c r="E453" s="44" t="s">
         <v>1990</v>
       </c>
-      <c r="F453" s="123"/>
-      <c r="G453" s="117"/>
+      <c r="F453" s="117"/>
+      <c r="G453" s="116"/>
     </row>
     <row r="454" spans="1:7">
       <c r="A454" s="44"/>
@@ -30233,8 +30233,8 @@
       <c r="E454" s="44" t="s">
         <v>1992</v>
       </c>
-      <c r="F454" s="123"/>
-      <c r="G454" s="117"/>
+      <c r="F454" s="117"/>
+      <c r="G454" s="116"/>
     </row>
     <row r="455" spans="1:7">
       <c r="A455" s="44"/>
@@ -30246,8 +30246,8 @@
       </c>
       <c r="D455" s="44"/>
       <c r="E455" s="44"/>
-      <c r="F455" s="123"/>
-      <c r="G455" s="117"/>
+      <c r="F455" s="117"/>
+      <c r="G455" s="116"/>
     </row>
     <row r="456" spans="1:7">
       <c r="A456" s="44"/>
@@ -30259,8 +30259,8 @@
       </c>
       <c r="D456" s="44"/>
       <c r="E456" s="44"/>
-      <c r="F456" s="123"/>
-      <c r="G456" s="117"/>
+      <c r="F456" s="117"/>
+      <c r="G456" s="116"/>
     </row>
     <row r="457" spans="1:7">
       <c r="A457" s="44"/>
@@ -30272,8 +30272,8 @@
       </c>
       <c r="D457" s="44"/>
       <c r="E457" s="44"/>
-      <c r="F457" s="123"/>
-      <c r="G457" s="117"/>
+      <c r="F457" s="117"/>
+      <c r="G457" s="116"/>
     </row>
     <row r="458" spans="1:7">
       <c r="A458" s="44"/>
@@ -30285,8 +30285,8 @@
       </c>
       <c r="D458" s="44"/>
       <c r="E458" s="44"/>
-      <c r="F458" s="123"/>
-      <c r="G458" s="117"/>
+      <c r="F458" s="117"/>
+      <c r="G458" s="116"/>
     </row>
     <row r="459" spans="1:7">
       <c r="A459" s="44"/>
@@ -30298,8 +30298,8 @@
       </c>
       <c r="D459" s="44"/>
       <c r="E459" s="44"/>
-      <c r="F459" s="123"/>
-      <c r="G459" s="117"/>
+      <c r="F459" s="117"/>
+      <c r="G459" s="116"/>
     </row>
     <row r="460" spans="1:7">
       <c r="A460" s="44"/>
@@ -30311,8 +30311,8 @@
       </c>
       <c r="D460" s="44"/>
       <c r="E460" s="44"/>
-      <c r="F460" s="123"/>
-      <c r="G460" s="117"/>
+      <c r="F460" s="117"/>
+      <c r="G460" s="116"/>
     </row>
     <row r="461" spans="1:7">
       <c r="A461" s="44"/>
@@ -30324,8 +30324,8 @@
       <c r="E461" s="44" t="s">
         <v>2006</v>
       </c>
-      <c r="F461" s="123"/>
-      <c r="G461" s="117"/>
+      <c r="F461" s="117"/>
+      <c r="G461" s="116"/>
     </row>
     <row r="462" spans="1:7">
       <c r="A462" s="44"/>
@@ -30337,8 +30337,8 @@
       <c r="E462" s="44" t="s">
         <v>2008</v>
       </c>
-      <c r="F462" s="123"/>
-      <c r="G462" s="117"/>
+      <c r="F462" s="117"/>
+      <c r="G462" s="116"/>
     </row>
     <row r="463" spans="1:7">
       <c r="A463" s="44"/>
@@ -30354,8 +30354,8 @@
       <c r="E463" s="44" t="s">
         <v>2012</v>
       </c>
-      <c r="F463" s="123"/>
-      <c r="G463" s="117"/>
+      <c r="F463" s="117"/>
+      <c r="G463" s="116"/>
     </row>
     <row r="464" spans="1:7">
       <c r="A464" s="44"/>
@@ -30367,8 +30367,8 @@
       <c r="E464" s="44" t="s">
         <v>2014</v>
       </c>
-      <c r="F464" s="123"/>
-      <c r="G464" s="117"/>
+      <c r="F464" s="117"/>
+      <c r="G464" s="116"/>
     </row>
     <row r="465" spans="1:7">
       <c r="A465" s="44"/>
@@ -30380,8 +30380,8 @@
       </c>
       <c r="D465" s="44"/>
       <c r="E465" s="44"/>
-      <c r="F465" s="123"/>
-      <c r="G465" s="117"/>
+      <c r="F465" s="117"/>
+      <c r="G465" s="116"/>
     </row>
     <row r="466" spans="1:7">
       <c r="A466" s="44"/>
@@ -30393,8 +30393,8 @@
       </c>
       <c r="D466" s="44"/>
       <c r="E466" s="44"/>
-      <c r="F466" s="123"/>
-      <c r="G466" s="117"/>
+      <c r="F466" s="117"/>
+      <c r="G466" s="116"/>
     </row>
     <row r="467" spans="1:7">
       <c r="A467" s="44"/>
@@ -30406,8 +30406,8 @@
       </c>
       <c r="D467" s="44"/>
       <c r="E467" s="44"/>
-      <c r="F467" s="123"/>
-      <c r="G467" s="117"/>
+      <c r="F467" s="117"/>
+      <c r="G467" s="116"/>
     </row>
     <row r="468" spans="1:7">
       <c r="A468" s="44"/>
@@ -30419,8 +30419,8 @@
       </c>
       <c r="D468" s="44"/>
       <c r="E468" s="44"/>
-      <c r="F468" s="123"/>
-      <c r="G468" s="117"/>
+      <c r="F468" s="117"/>
+      <c r="G468" s="116"/>
     </row>
     <row r="469" spans="1:7">
       <c r="A469" s="44"/>
@@ -30432,8 +30432,8 @@
       </c>
       <c r="D469" s="44"/>
       <c r="E469" s="44"/>
-      <c r="F469" s="123"/>
-      <c r="G469" s="117"/>
+      <c r="F469" s="117"/>
+      <c r="G469" s="116"/>
     </row>
     <row r="470" spans="1:7">
       <c r="A470" s="44"/>
@@ -30445,8 +30445,8 @@
       </c>
       <c r="D470" s="44"/>
       <c r="E470" s="44"/>
-      <c r="F470" s="123"/>
-      <c r="G470" s="117"/>
+      <c r="F470" s="117"/>
+      <c r="G470" s="116"/>
     </row>
     <row r="471" spans="1:7">
       <c r="A471" s="44"/>
@@ -30458,8 +30458,8 @@
       </c>
       <c r="D471" s="44"/>
       <c r="E471" s="44"/>
-      <c r="F471" s="123"/>
-      <c r="G471" s="117"/>
+      <c r="F471" s="117"/>
+      <c r="G471" s="116"/>
     </row>
     <row r="472" spans="1:7">
       <c r="A472" s="44"/>
@@ -30471,8 +30471,8 @@
       </c>
       <c r="D472" s="44"/>
       <c r="E472" s="44"/>
-      <c r="F472" s="123"/>
-      <c r="G472" s="117"/>
+      <c r="F472" s="117"/>
+      <c r="G472" s="116"/>
     </row>
     <row r="473" spans="1:7">
       <c r="A473" s="44"/>
@@ -30484,8 +30484,8 @@
       </c>
       <c r="D473" s="44"/>
       <c r="E473" s="44"/>
-      <c r="F473" s="123"/>
-      <c r="G473" s="117"/>
+      <c r="F473" s="117"/>
+      <c r="G473" s="116"/>
     </row>
     <row r="474" spans="1:7">
       <c r="A474" s="44"/>
@@ -30501,7 +30501,7 @@
       <c r="E474" s="44" t="s">
         <v>2036</v>
       </c>
-      <c r="F474" s="123"/>
+      <c r="F474" s="117"/>
       <c r="G474" s="44"/>
     </row>
     <row r="475" spans="1:7">
@@ -30514,7 +30514,7 @@
       <c r="E475" s="44" t="s">
         <v>2038</v>
       </c>
-      <c r="F475" s="123"/>
+      <c r="F475" s="117"/>
       <c r="G475" s="44"/>
     </row>
     <row r="476" spans="1:7">
@@ -30523,7 +30523,7 @@
       <c r="C476" s="44"/>
       <c r="D476" s="44"/>
       <c r="E476" s="44"/>
-      <c r="F476" s="123"/>
+      <c r="F476" s="117"/>
       <c r="G476" s="44"/>
     </row>
     <row r="477" spans="1:7">
@@ -30695,22 +30695,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="F316:F318"/>
-    <mergeCell ref="G316:G318"/>
-    <mergeCell ref="F450:F476"/>
-    <mergeCell ref="G450:G473"/>
-    <mergeCell ref="F118:F119"/>
-    <mergeCell ref="G118:G119"/>
-    <mergeCell ref="F137:F139"/>
-    <mergeCell ref="G137:G139"/>
-    <mergeCell ref="F279:F295"/>
-    <mergeCell ref="G279:G295"/>
-    <mergeCell ref="F2:F6"/>
-    <mergeCell ref="G2:G6"/>
-    <mergeCell ref="F7:F13"/>
-    <mergeCell ref="G7:G13"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="G14:G18"/>
     <mergeCell ref="F19:F23"/>
     <mergeCell ref="G19:G23"/>
     <mergeCell ref="F304:F308"/>
@@ -30727,6 +30711,22 @@
     <mergeCell ref="G25:G31"/>
     <mergeCell ref="F64:F88"/>
     <mergeCell ref="G64:G88"/>
+    <mergeCell ref="F2:F6"/>
+    <mergeCell ref="G2:G6"/>
+    <mergeCell ref="F7:F13"/>
+    <mergeCell ref="G7:G13"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="G14:G18"/>
+    <mergeCell ref="F316:F318"/>
+    <mergeCell ref="G316:G318"/>
+    <mergeCell ref="F450:F476"/>
+    <mergeCell ref="G450:G473"/>
+    <mergeCell ref="F118:F119"/>
+    <mergeCell ref="G118:G119"/>
+    <mergeCell ref="F137:F139"/>
+    <mergeCell ref="G137:G139"/>
+    <mergeCell ref="F279:F295"/>
+    <mergeCell ref="G279:G295"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -31670,52 +31670,11 @@
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -32007,11 +31966,52 @@
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -32033,9 +32033,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -32061,9 +32061,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>